<commit_message>
Add total AOI column to configuration workbook
</commit_message>
<xml_diff>
--- a/v2/round100/V2配置点位与像面.xlsx
+++ b/v2/round100/V2配置点位与像面.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配置查询" sheetId="1" r:id="Rde4e72adb1df4d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部配置" sheetId="2" r:id="R288bf13763724cf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配置查询" sheetId="1" r:id="Re04d065ea0244fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部配置" sheetId="2" r:id="R5f04595757004e20"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -182,9 +182,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="V2Configurations" displayName="V2Configurations" ref="A7:R167" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:R167"/>
-  <x:tableColumns count="18">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="V2Configurations" displayName="V2Configurations" ref="A7:S167" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:S167"/>
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="配置号"/>
     <x:tableColumn id="2" name="点位编号"/>
     <x:tableColumn id="3" name="配置类型"/>
@@ -203,6 +203,7 @@
     <x:tableColumn id="16" name="像面全局 Z / mm"/>
     <x:tableColumn id="17" name="像面相对中面Z / mm"/>
     <x:tableColumn id="18" name="像面朝向"/>
+    <x:tableColumn id="19" name="总 AOI / °"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -570,17 +571,17 @@
     </x:row>
     <x:row r="14" ht="26" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>总入射角</x:v>
+        <x:v>总 AOI</x:v>
       </x:c>
       <x:c r="B14" s="17" t="n">
-        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(B12))^2+TAN(RADIANS(B13))^2)))</x:f>
-        <x:v>7.499999999999999</x:v>
+        <x:f>ROUND(INDEX('全部配置'!$S$8:$S$167,$D$4),9)</x:f>
+        <x:v>7.5</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
         <x:v>°</x:v>
       </x:c>
       <x:c r="D14" s="8" t="str">
-        <x:v>由 α、β 换算，不直接相加</x:v>
+        <x:v>相对工件Z法线，由α、β计算</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
@@ -765,6 +766,7 @@
     <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -880,7 +882,9 @@
       <x:c r="R5" s="2"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="2"/>
+      <x:c r="A6" s="8" t="str">
+        <x:v>AOI为光束与工件Z法线的夹角，由α、β计算；与像面朝向分开记录。</x:v>
+      </x:c>
       <x:c r="B6" s="2"/>
       <x:c r="C6" s="2"/>
       <x:c r="D6" s="2"/>
@@ -954,6 +958,9 @@
       <x:c r="R7" s="22" t="str">
         <x:v>像面朝向</x:v>
       </x:c>
+      <x:c r="S7" s="22" t="str">
+        <x:v>总 AOI / °</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="24" t="n">
@@ -1011,6 +1018,10 @@
       <x:c r="R8" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S8" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G8))^2+TAN(RADIANS(H8))^2)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="24" t="n">
@@ -1068,6 +1079,10 @@
       <x:c r="R9" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S9" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G9))^2+TAN(RADIANS(H9))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="24" t="n">
@@ -1125,6 +1140,10 @@
       <x:c r="R10" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S10" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G10))^2+TAN(RADIANS(H10))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="24" t="n">
@@ -1182,6 +1201,10 @@
       <x:c r="R11" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S11" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G11))^2+TAN(RADIANS(H11))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="24" t="n">
@@ -1239,6 +1262,10 @@
       <x:c r="R12" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S12" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G12))^2+TAN(RADIANS(H12))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="24" t="n">
@@ -1296,6 +1323,10 @@
       <x:c r="R13" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S13" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G13))^2+TAN(RADIANS(H13))^2)))</x:f>
+        <x:v>1.5000000000000002</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="24" t="n">
@@ -1353,6 +1384,10 @@
       <x:c r="R14" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S14" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G14))^2+TAN(RADIANS(H14))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="24" t="n">
@@ -1410,6 +1445,10 @@
       <x:c r="R15" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S15" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G15))^2+TAN(RADIANS(H15))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="24" t="n">
@@ -1467,6 +1506,10 @@
       <x:c r="R16" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S16" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G16))^2+TAN(RADIANS(H16))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="24" t="n">
@@ -1524,6 +1567,10 @@
       <x:c r="R17" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S17" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G17))^2+TAN(RADIANS(H17))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="24" t="n">
@@ -1581,6 +1628,10 @@
       <x:c r="R18" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S18" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G18))^2+TAN(RADIANS(H18))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="24" t="n">
@@ -1638,6 +1689,10 @@
       <x:c r="R19" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S19" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G19))^2+TAN(RADIANS(H19))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="24" t="n">
@@ -1695,6 +1750,10 @@
       <x:c r="R20" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S20" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G20))^2+TAN(RADIANS(H20))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="24" t="n">
@@ -1752,6 +1811,10 @@
       <x:c r="R21" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S21" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G21))^2+TAN(RADIANS(H21))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="24" t="n">
@@ -1809,6 +1872,10 @@
       <x:c r="R22" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S22" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G22))^2+TAN(RADIANS(H22))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="24" t="n">
@@ -1866,6 +1933,10 @@
       <x:c r="R23" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S23" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G23))^2+TAN(RADIANS(H23))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="24" t="n">
@@ -1923,6 +1994,10 @@
       <x:c r="R24" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S24" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G24))^2+TAN(RADIANS(H24))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="24" t="n">
@@ -1980,6 +2055,10 @@
       <x:c r="R25" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S25" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G25))^2+TAN(RADIANS(H25))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="24" t="n">
@@ -2037,6 +2116,10 @@
       <x:c r="R26" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S26" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G26))^2+TAN(RADIANS(H26))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="24" t="n">
@@ -2094,6 +2177,10 @@
       <x:c r="R27" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S27" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G27))^2+TAN(RADIANS(H27))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="24" t="n">
@@ -2151,6 +2238,10 @@
       <x:c r="R28" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S28" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G28))^2+TAN(RADIANS(H28))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="24" t="n">
@@ -2208,6 +2299,10 @@
       <x:c r="R29" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S29" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G29))^2+TAN(RADIANS(H29))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="24" t="n">
@@ -2265,6 +2360,10 @@
       <x:c r="R30" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S30" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G30))^2+TAN(RADIANS(H30))^2)))</x:f>
+        <x:v>1.5000000000000002</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="24" t="n">
@@ -2322,6 +2421,10 @@
       <x:c r="R31" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S31" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G31))^2+TAN(RADIANS(H31))^2)))</x:f>
+        <x:v>1.5000000000000002</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="24" t="n">
@@ -2379,6 +2482,10 @@
       <x:c r="R32" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S32" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G32))^2+TAN(RADIANS(H32))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="24" t="n">
@@ -2436,6 +2543,10 @@
       <x:c r="R33" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S33" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G33))^2+TAN(RADIANS(H33))^2)))</x:f>
+        <x:v>1.4999999999999998</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="24" t="n">
@@ -2493,6 +2604,10 @@
       <x:c r="R34" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S34" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G34))^2+TAN(RADIANS(H34))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="24" t="n">
@@ -2550,6 +2665,10 @@
       <x:c r="R35" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S35" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G35))^2+TAN(RADIANS(H35))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="24" t="n">
@@ -2607,6 +2726,10 @@
       <x:c r="R36" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S36" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G36))^2+TAN(RADIANS(H36))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
       <x:c r="A37" s="24" t="n">
@@ -2664,6 +2787,10 @@
       <x:c r="R37" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S37" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G37))^2+TAN(RADIANS(H37))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="24" t="n">
@@ -2721,6 +2848,10 @@
       <x:c r="R38" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S38" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G38))^2+TAN(RADIANS(H38))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
       <x:c r="A39" s="24" t="n">
@@ -2778,6 +2909,10 @@
       <x:c r="R39" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S39" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G39))^2+TAN(RADIANS(H39))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="24" t="n">
@@ -2835,6 +2970,10 @@
       <x:c r="R40" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S40" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G40))^2+TAN(RADIANS(H40))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="A41" s="24" t="n">
@@ -2892,6 +3031,10 @@
       <x:c r="R41" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S41" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G41))^2+TAN(RADIANS(H41))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
       <x:c r="A42" s="24" t="n">
@@ -2949,6 +3092,10 @@
       <x:c r="R42" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S42" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G42))^2+TAN(RADIANS(H42))^2)))</x:f>
+        <x:v>1.5000000000000002</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
       <x:c r="A43" s="24" t="n">
@@ -3006,6 +3153,10 @@
       <x:c r="R43" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S43" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G43))^2+TAN(RADIANS(H43))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="24" t="n">
@@ -3063,6 +3214,10 @@
       <x:c r="R44" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S44" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G44))^2+TAN(RADIANS(H44))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
       <x:c r="A45" s="24" t="n">
@@ -3120,6 +3275,10 @@
       <x:c r="R45" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S45" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G45))^2+TAN(RADIANS(H45))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
       <x:c r="A46" s="24" t="n">
@@ -3177,6 +3336,10 @@
       <x:c r="R46" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S46" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G46))^2+TAN(RADIANS(H46))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
       <x:c r="A47" s="24" t="n">
@@ -3234,6 +3397,10 @@
       <x:c r="R47" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S47" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G47))^2+TAN(RADIANS(H47))^2)))</x:f>
+        <x:v>1.5000000000000002</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
       <x:c r="A48" s="24" t="n">
@@ -3291,6 +3458,10 @@
       <x:c r="R48" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S48" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G48))^2+TAN(RADIANS(H48))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
       <x:c r="A49" s="24" t="n">
@@ -3348,6 +3519,10 @@
       <x:c r="R49" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S49" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G49))^2+TAN(RADIANS(H49))^2)))</x:f>
+        <x:v>1.5000000000000002</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
       <x:c r="A50" s="24" t="n">
@@ -3405,6 +3580,10 @@
       <x:c r="R50" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S50" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G50))^2+TAN(RADIANS(H50))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
       <x:c r="A51" s="24" t="n">
@@ -3462,6 +3641,10 @@
       <x:c r="R51" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S51" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G51))^2+TAN(RADIANS(H51))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
       <x:c r="A52" s="24" t="n">
@@ -3519,6 +3702,10 @@
       <x:c r="R52" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S52" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G52))^2+TAN(RADIANS(H52))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
       <x:c r="A53" s="24" t="n">
@@ -3576,6 +3763,10 @@
       <x:c r="R53" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S53" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G53))^2+TAN(RADIANS(H53))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
       <x:c r="A54" s="24" t="n">
@@ -3633,6 +3824,10 @@
       <x:c r="R54" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S54" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G54))^2+TAN(RADIANS(H54))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
       <x:c r="A55" s="24" t="n">
@@ -3690,6 +3885,10 @@
       <x:c r="R55" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S55" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G55))^2+TAN(RADIANS(H55))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
       <x:c r="A56" s="24" t="n">
@@ -3747,6 +3946,10 @@
       <x:c r="R56" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S56" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G56))^2+TAN(RADIANS(H56))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
       <x:c r="A57" s="24" t="n">
@@ -3804,6 +4007,10 @@
       <x:c r="R57" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S57" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G57))^2+TAN(RADIANS(H57))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
       <x:c r="A58" s="24" t="n">
@@ -3861,6 +4068,10 @@
       <x:c r="R58" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S58" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G58))^2+TAN(RADIANS(H58))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
       <x:c r="A59" s="24" t="n">
@@ -3918,6 +4129,10 @@
       <x:c r="R59" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S59" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G59))^2+TAN(RADIANS(H59))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
       <x:c r="A60" s="24" t="n">
@@ -3975,6 +4190,10 @@
       <x:c r="R60" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S60" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G60))^2+TAN(RADIANS(H60))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
       <x:c r="A61" s="24" t="n">
@@ -4032,6 +4251,10 @@
       <x:c r="R61" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S61" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G61))^2+TAN(RADIANS(H61))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
       <x:c r="A62" s="24" t="n">
@@ -4089,6 +4312,10 @@
       <x:c r="R62" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S62" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G62))^2+TAN(RADIANS(H62))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
       <x:c r="A63" s="24" t="n">
@@ -4146,6 +4373,10 @@
       <x:c r="R63" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S63" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G63))^2+TAN(RADIANS(H63))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
       <x:c r="A64" s="24" t="n">
@@ -4203,6 +4434,10 @@
       <x:c r="R64" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S64" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G64))^2+TAN(RADIANS(H64))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="24" customHeight="1">
       <x:c r="A65" s="24" t="n">
@@ -4260,6 +4495,10 @@
       <x:c r="R65" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S65" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G65))^2+TAN(RADIANS(H65))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="24" customHeight="1">
       <x:c r="A66" s="24" t="n">
@@ -4317,6 +4556,10 @@
       <x:c r="R66" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S66" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G66))^2+TAN(RADIANS(H66))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="24" customHeight="1">
       <x:c r="A67" s="24" t="n">
@@ -4374,6 +4617,10 @@
       <x:c r="R67" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S67" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G67))^2+TAN(RADIANS(H67))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
       <x:c r="A68" s="24" t="n">
@@ -4431,6 +4678,10 @@
       <x:c r="R68" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S68" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G68))^2+TAN(RADIANS(H68))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="24" customHeight="1">
       <x:c r="A69" s="24" t="n">
@@ -4488,6 +4739,10 @@
       <x:c r="R69" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S69" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G69))^2+TAN(RADIANS(H69))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="24" customHeight="1">
       <x:c r="A70" s="24" t="n">
@@ -4545,6 +4800,10 @@
       <x:c r="R70" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S70" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G70))^2+TAN(RADIANS(H70))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
       <x:c r="A71" s="24" t="n">
@@ -4602,6 +4861,10 @@
       <x:c r="R71" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S71" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G71))^2+TAN(RADIANS(H71))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="24" customHeight="1">
       <x:c r="A72" s="24" t="n">
@@ -4659,6 +4922,10 @@
       <x:c r="R72" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S72" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G72))^2+TAN(RADIANS(H72))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="24" customHeight="1">
       <x:c r="A73" s="24" t="n">
@@ -4716,6 +4983,10 @@
       <x:c r="R73" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S73" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G73))^2+TAN(RADIANS(H73))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
       <x:c r="A74" s="24" t="n">
@@ -4773,6 +5044,10 @@
       <x:c r="R74" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S74" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G74))^2+TAN(RADIANS(H74))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="24" customHeight="1">
       <x:c r="A75" s="24" t="n">
@@ -4830,6 +5105,10 @@
       <x:c r="R75" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S75" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G75))^2+TAN(RADIANS(H75))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="24" customHeight="1">
       <x:c r="A76" s="24" t="n">
@@ -4887,6 +5166,10 @@
       <x:c r="R76" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S76" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G76))^2+TAN(RADIANS(H76))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="24" customHeight="1">
       <x:c r="A77" s="24" t="n">
@@ -4944,6 +5227,10 @@
       <x:c r="R77" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S77" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G77))^2+TAN(RADIANS(H77))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
       <x:c r="A78" s="24" t="n">
@@ -5001,6 +5288,10 @@
       <x:c r="R78" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S78" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G78))^2+TAN(RADIANS(H78))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="24" customHeight="1">
       <x:c r="A79" s="24" t="n">
@@ -5058,6 +5349,10 @@
       <x:c r="R79" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S79" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G79))^2+TAN(RADIANS(H79))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="24" customHeight="1">
       <x:c r="A80" s="24" t="n">
@@ -5115,6 +5410,10 @@
       <x:c r="R80" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S80" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G80))^2+TAN(RADIANS(H80))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" ht="24" customHeight="1">
       <x:c r="A81" s="24" t="n">
@@ -5172,6 +5471,10 @@
       <x:c r="R81" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S81" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G81))^2+TAN(RADIANS(H81))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="24" customHeight="1">
       <x:c r="A82" s="24" t="n">
@@ -5229,6 +5532,10 @@
       <x:c r="R82" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S82" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G82))^2+TAN(RADIANS(H82))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="24" customHeight="1">
       <x:c r="A83" s="24" t="n">
@@ -5286,6 +5593,10 @@
       <x:c r="R83" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S83" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G83))^2+TAN(RADIANS(H83))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="24" customHeight="1">
       <x:c r="A84" s="24" t="n">
@@ -5343,6 +5654,10 @@
       <x:c r="R84" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S84" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G84))^2+TAN(RADIANS(H84))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="24" customHeight="1">
       <x:c r="A85" s="24" t="n">
@@ -5400,6 +5715,10 @@
       <x:c r="R85" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S85" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G85))^2+TAN(RADIANS(H85))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="24" customHeight="1">
       <x:c r="A86" s="24" t="n">
@@ -5457,6 +5776,10 @@
       <x:c r="R86" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S86" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G86))^2+TAN(RADIANS(H86))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="24" customHeight="1">
       <x:c r="A87" s="24" t="n">
@@ -5514,6 +5837,10 @@
       <x:c r="R87" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S87" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G87))^2+TAN(RADIANS(H87))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="24" customHeight="1">
       <x:c r="A88" s="24" t="n">
@@ -5571,6 +5898,10 @@
       <x:c r="R88" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S88" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G88))^2+TAN(RADIANS(H88))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="24" customHeight="1">
       <x:c r="A89" s="24" t="n">
@@ -5628,6 +5959,10 @@
       <x:c r="R89" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S89" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G89))^2+TAN(RADIANS(H89))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="24" customHeight="1">
       <x:c r="A90" s="24" t="n">
@@ -5685,6 +6020,10 @@
       <x:c r="R90" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S90" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G90))^2+TAN(RADIANS(H90))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="24" customHeight="1">
       <x:c r="A91" s="24" t="n">
@@ -5742,6 +6081,10 @@
       <x:c r="R91" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S91" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G91))^2+TAN(RADIANS(H91))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="92" ht="24" customHeight="1">
       <x:c r="A92" s="24" t="n">
@@ -5799,6 +6142,10 @@
       <x:c r="R92" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S92" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G92))^2+TAN(RADIANS(H92))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="93" ht="24" customHeight="1">
       <x:c r="A93" s="24" t="n">
@@ -5856,6 +6203,10 @@
       <x:c r="R93" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S93" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G93))^2+TAN(RADIANS(H93))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" ht="24" customHeight="1">
       <x:c r="A94" s="24" t="n">
@@ -5913,6 +6264,10 @@
       <x:c r="R94" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S94" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G94))^2+TAN(RADIANS(H94))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="95" ht="24" customHeight="1">
       <x:c r="A95" s="24" t="n">
@@ -5970,6 +6325,10 @@
       <x:c r="R95" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S95" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G95))^2+TAN(RADIANS(H95))^2)))</x:f>
+        <x:v>1.5000000000000002</x:v>
+      </x:c>
     </x:row>
     <x:row r="96" ht="24" customHeight="1">
       <x:c r="A96" s="24" t="n">
@@ -6027,6 +6386,10 @@
       <x:c r="R96" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S96" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G96))^2+TAN(RADIANS(H96))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="97" ht="24" customHeight="1">
       <x:c r="A97" s="24" t="n">
@@ -6084,6 +6447,10 @@
       <x:c r="R97" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S97" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G97))^2+TAN(RADIANS(H97))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
       <x:c r="A98" s="24" t="n">
@@ -6141,6 +6508,10 @@
       <x:c r="R98" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S98" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G98))^2+TAN(RADIANS(H98))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="99" ht="24" customHeight="1">
       <x:c r="A99" s="24" t="n">
@@ -6198,6 +6569,10 @@
       <x:c r="R99" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S99" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G99))^2+TAN(RADIANS(H99))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="100" ht="24" customHeight="1">
       <x:c r="A100" s="24" t="n">
@@ -6255,6 +6630,10 @@
       <x:c r="R100" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S100" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G100))^2+TAN(RADIANS(H100))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="101" ht="24" customHeight="1">
       <x:c r="A101" s="24" t="n">
@@ -6312,6 +6691,10 @@
       <x:c r="R101" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S101" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G101))^2+TAN(RADIANS(H101))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="102" ht="24" customHeight="1">
       <x:c r="A102" s="24" t="n">
@@ -6369,6 +6752,10 @@
       <x:c r="R102" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S102" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G102))^2+TAN(RADIANS(H102))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="103" ht="24" customHeight="1">
       <x:c r="A103" s="24" t="n">
@@ -6426,6 +6813,10 @@
       <x:c r="R103" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S103" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G103))^2+TAN(RADIANS(H103))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="104" ht="24" customHeight="1">
       <x:c r="A104" s="24" t="n">
@@ -6483,6 +6874,10 @@
       <x:c r="R104" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S104" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G104))^2+TAN(RADIANS(H104))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="105" ht="24" customHeight="1">
       <x:c r="A105" s="24" t="n">
@@ -6540,6 +6935,10 @@
       <x:c r="R105" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S105" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G105))^2+TAN(RADIANS(H105))^2)))</x:f>
+        <x:v>1.5000000000000002</x:v>
+      </x:c>
     </x:row>
     <x:row r="106" ht="24" customHeight="1">
       <x:c r="A106" s="24" t="n">
@@ -6597,6 +6996,10 @@
       <x:c r="R106" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S106" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G106))^2+TAN(RADIANS(H106))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="107" ht="24" customHeight="1">
       <x:c r="A107" s="24" t="n">
@@ -6654,6 +7057,10 @@
       <x:c r="R107" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S107" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G107))^2+TAN(RADIANS(H107))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="108" ht="24" customHeight="1">
       <x:c r="A108" s="24" t="n">
@@ -6711,6 +7118,10 @@
       <x:c r="R108" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S108" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G108))^2+TAN(RADIANS(H108))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="109" ht="24" customHeight="1">
       <x:c r="A109" s="24" t="n">
@@ -6768,6 +7179,10 @@
       <x:c r="R109" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S109" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G109))^2+TAN(RADIANS(H109))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="110" ht="24" customHeight="1">
       <x:c r="A110" s="24" t="n">
@@ -6825,6 +7240,10 @@
       <x:c r="R110" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S110" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G110))^2+TAN(RADIANS(H110))^2)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="111" ht="24" customHeight="1">
       <x:c r="A111" s="24" t="n">
@@ -6882,6 +7301,10 @@
       <x:c r="R111" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S111" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G111))^2+TAN(RADIANS(H111))^2)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="112" ht="24" customHeight="1">
       <x:c r="A112" s="24" t="n">
@@ -6939,6 +7362,10 @@
       <x:c r="R112" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S112" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G112))^2+TAN(RADIANS(H112))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="113" ht="24" customHeight="1">
       <x:c r="A113" s="24" t="n">
@@ -6996,6 +7423,10 @@
       <x:c r="R113" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S113" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G113))^2+TAN(RADIANS(H113))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="114" ht="24" customHeight="1">
       <x:c r="A114" s="24" t="n">
@@ -7053,6 +7484,10 @@
       <x:c r="R114" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S114" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G114))^2+TAN(RADIANS(H114))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="115" ht="24" customHeight="1">
       <x:c r="A115" s="24" t="n">
@@ -7110,6 +7545,10 @@
       <x:c r="R115" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S115" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G115))^2+TAN(RADIANS(H115))^2)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="116" ht="24" customHeight="1">
       <x:c r="A116" s="24" t="n">
@@ -7167,6 +7606,10 @@
       <x:c r="R116" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S116" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G116))^2+TAN(RADIANS(H116))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="117" ht="24" customHeight="1">
       <x:c r="A117" s="24" t="n">
@@ -7224,6 +7667,10 @@
       <x:c r="R117" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S117" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G117))^2+TAN(RADIANS(H117))^2)))</x:f>
+        <x:v>5.000000000000001</x:v>
+      </x:c>
     </x:row>
     <x:row r="118" ht="24" customHeight="1">
       <x:c r="A118" s="24" t="n">
@@ -7281,6 +7728,10 @@
       <x:c r="R118" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S118" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G118))^2+TAN(RADIANS(H118))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="119" ht="24" customHeight="1">
       <x:c r="A119" s="24" t="n">
@@ -7338,6 +7789,10 @@
       <x:c r="R119" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S119" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G119))^2+TAN(RADIANS(H119))^2)))</x:f>
+        <x:v>5.000000000000001</x:v>
+      </x:c>
     </x:row>
     <x:row r="120" ht="24" customHeight="1">
       <x:c r="A120" s="24" t="n">
@@ -7395,6 +7850,10 @@
       <x:c r="R120" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S120" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G120))^2+TAN(RADIANS(H120))^2)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="121" ht="24" customHeight="1">
       <x:c r="A121" s="24" t="n">
@@ -7452,6 +7911,10 @@
       <x:c r="R121" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S121" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G121))^2+TAN(RADIANS(H121))^2)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="122" ht="24" customHeight="1">
       <x:c r="A122" s="24" t="n">
@@ -7509,6 +7972,10 @@
       <x:c r="R122" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S122" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G122))^2+TAN(RADIANS(H122))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="123" ht="24" customHeight="1">
       <x:c r="A123" s="24" t="n">
@@ -7566,6 +8033,10 @@
       <x:c r="R123" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S123" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G123))^2+TAN(RADIANS(H123))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="124" ht="24" customHeight="1">
       <x:c r="A124" s="24" t="n">
@@ -7623,6 +8094,10 @@
       <x:c r="R124" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S124" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G124))^2+TAN(RADIANS(H124))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="125" ht="24" customHeight="1">
       <x:c r="A125" s="24" t="n">
@@ -7680,6 +8155,10 @@
       <x:c r="R125" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S125" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G125))^2+TAN(RADIANS(H125))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="126" ht="24" customHeight="1">
       <x:c r="A126" s="24" t="n">
@@ -7737,6 +8216,10 @@
       <x:c r="R126" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S126" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G126))^2+TAN(RADIANS(H126))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="127" ht="24" customHeight="1">
       <x:c r="A127" s="24" t="n">
@@ -7794,6 +8277,10 @@
       <x:c r="R127" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S127" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G127))^2+TAN(RADIANS(H127))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="128" ht="24" customHeight="1">
       <x:c r="A128" s="24" t="n">
@@ -7851,6 +8338,10 @@
       <x:c r="R128" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S128" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G128))^2+TAN(RADIANS(H128))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="129" ht="24" customHeight="1">
       <x:c r="A129" s="24" t="n">
@@ -7908,6 +8399,10 @@
       <x:c r="R129" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S129" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G129))^2+TAN(RADIANS(H129))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="130" ht="24" customHeight="1">
       <x:c r="A130" s="24" t="n">
@@ -7965,6 +8460,10 @@
       <x:c r="R130" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S130" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G130))^2+TAN(RADIANS(H130))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="131" ht="24" customHeight="1">
       <x:c r="A131" s="24" t="n">
@@ -8022,6 +8521,10 @@
       <x:c r="R131" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S131" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G131))^2+TAN(RADIANS(H131))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="132" ht="24" customHeight="1">
       <x:c r="A132" s="24" t="n">
@@ -8079,6 +8582,10 @@
       <x:c r="R132" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S132" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G132))^2+TAN(RADIANS(H132))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="133" ht="24" customHeight="1">
       <x:c r="A133" s="24" t="n">
@@ -8136,6 +8643,10 @@
       <x:c r="R133" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S133" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G133))^2+TAN(RADIANS(H133))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="134" ht="24" customHeight="1">
       <x:c r="A134" s="24" t="n">
@@ -8193,6 +8704,10 @@
       <x:c r="R134" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S134" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G134))^2+TAN(RADIANS(H134))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="135" ht="24" customHeight="1">
       <x:c r="A135" s="24" t="n">
@@ -8250,6 +8765,10 @@
       <x:c r="R135" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S135" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G135))^2+TAN(RADIANS(H135))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="136" ht="24" customHeight="1">
       <x:c r="A136" s="24" t="n">
@@ -8307,6 +8826,10 @@
       <x:c r="R136" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S136" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G136))^2+TAN(RADIANS(H136))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="137" ht="24" customHeight="1">
       <x:c r="A137" s="24" t="n">
@@ -8364,6 +8887,10 @@
       <x:c r="R137" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S137" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G137))^2+TAN(RADIANS(H137))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="138" ht="24" customHeight="1">
       <x:c r="A138" s="24" t="n">
@@ -8421,6 +8948,10 @@
       <x:c r="R138" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S138" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G138))^2+TAN(RADIANS(H138))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="139" ht="24" customHeight="1">
       <x:c r="A139" s="24" t="n">
@@ -8478,6 +9009,10 @@
       <x:c r="R139" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S139" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G139))^2+TAN(RADIANS(H139))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="140" ht="24" customHeight="1">
       <x:c r="A140" s="24" t="n">
@@ -8535,6 +9070,10 @@
       <x:c r="R140" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S140" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G140))^2+TAN(RADIANS(H140))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="141" ht="24" customHeight="1">
       <x:c r="A141" s="24" t="n">
@@ -8592,6 +9131,10 @@
       <x:c r="R141" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S141" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G141))^2+TAN(RADIANS(H141))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="142" ht="24" customHeight="1">
       <x:c r="A142" s="24" t="n">
@@ -8649,6 +9192,10 @@
       <x:c r="R142" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S142" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G142))^2+TAN(RADIANS(H142))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="143" ht="24" customHeight="1">
       <x:c r="A143" s="24" t="n">
@@ -8706,6 +9253,10 @@
       <x:c r="R143" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S143" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G143))^2+TAN(RADIANS(H143))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="144" ht="24" customHeight="1">
       <x:c r="A144" s="24" t="n">
@@ -8763,6 +9314,10 @@
       <x:c r="R144" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S144" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G144))^2+TAN(RADIANS(H144))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="145" ht="24" customHeight="1">
       <x:c r="A145" s="24" t="n">
@@ -8820,6 +9375,10 @@
       <x:c r="R145" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S145" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G145))^2+TAN(RADIANS(H145))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="146" ht="24" customHeight="1">
       <x:c r="A146" s="24" t="n">
@@ -8877,6 +9436,10 @@
       <x:c r="R146" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S146" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G146))^2+TAN(RADIANS(H146))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="147" ht="24" customHeight="1">
       <x:c r="A147" s="24" t="n">
@@ -8934,6 +9497,10 @@
       <x:c r="R147" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S147" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G147))^2+TAN(RADIANS(H147))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="148" ht="24" customHeight="1">
       <x:c r="A148" s="24" t="n">
@@ -8991,6 +9558,10 @@
       <x:c r="R148" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S148" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G148))^2+TAN(RADIANS(H148))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="149" ht="24" customHeight="1">
       <x:c r="A149" s="24" t="n">
@@ -9048,6 +9619,10 @@
       <x:c r="R149" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S149" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G149))^2+TAN(RADIANS(H149))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="150" ht="24" customHeight="1">
       <x:c r="A150" s="24" t="n">
@@ -9105,6 +9680,10 @@
       <x:c r="R150" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S150" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G150))^2+TAN(RADIANS(H150))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="151" ht="24" customHeight="1">
       <x:c r="A151" s="24" t="n">
@@ -9162,6 +9741,10 @@
       <x:c r="R151" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S151" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G151))^2+TAN(RADIANS(H151))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="152" ht="24" customHeight="1">
       <x:c r="A152" s="24" t="n">
@@ -9219,6 +9802,10 @@
       <x:c r="R152" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S152" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G152))^2+TAN(RADIANS(H152))^2)))</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="153" ht="24" customHeight="1">
       <x:c r="A153" s="24" t="n">
@@ -9276,6 +9863,10 @@
       <x:c r="R153" s="2" t="str">
         <x:v>垂直末端主光线</x:v>
       </x:c>
+      <x:c r="S153" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G153))^2+TAN(RADIANS(H153))^2)))</x:f>
+        <x:v>7.499999999999999</x:v>
+      </x:c>
     </x:row>
     <x:row r="154" ht="24" customHeight="1">
       <x:c r="A154" s="24" t="n">
@@ -9333,6 +9924,10 @@
       <x:c r="R154" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S154" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G154))^2+TAN(RADIANS(H154))^2)))</x:f>
+        <x:v>3.0000000000000004</x:v>
+      </x:c>
     </x:row>
     <x:row r="155" ht="24" customHeight="1">
       <x:c r="A155" s="24" t="n">
@@ -9390,6 +9985,10 @@
       <x:c r="R155" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S155" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G155))^2+TAN(RADIANS(H155))^2)))</x:f>
+        <x:v>3.0000000000000013</x:v>
+      </x:c>
     </x:row>
     <x:row r="156" ht="24" customHeight="1">
       <x:c r="A156" s="24" t="n">
@@ -9447,6 +10046,10 @@
       <x:c r="R156" s="2" t="str">
         <x:v>垂直末端主光线</x:v>
       </x:c>
+      <x:c r="S156" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G156))^2+TAN(RADIANS(H156))^2)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="157" ht="24" customHeight="1">
       <x:c r="A157" s="24" t="n">
@@ -9504,6 +10107,10 @@
       <x:c r="R157" s="2" t="str">
         <x:v>垂直末端主光线</x:v>
       </x:c>
+      <x:c r="S157" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G157))^2+TAN(RADIANS(H157))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="158" ht="24" customHeight="1">
       <x:c r="A158" s="24" t="n">
@@ -9561,6 +10168,10 @@
       <x:c r="R158" s="2" t="str">
         <x:v>垂直末端主光线</x:v>
       </x:c>
+      <x:c r="S158" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G158))^2+TAN(RADIANS(H158))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="159" ht="24" customHeight="1">
       <x:c r="A159" s="24" t="n">
@@ -9618,6 +10229,10 @@
       <x:c r="R159" s="2" t="str">
         <x:v>垂直末端主光线</x:v>
       </x:c>
+      <x:c r="S159" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G159))^2+TAN(RADIANS(H159))^2)))</x:f>
+        <x:v>7.499999999999999</x:v>
+      </x:c>
     </x:row>
     <x:row r="160" ht="24" customHeight="1">
       <x:c r="A160" s="24" t="n">
@@ -9675,6 +10290,10 @@
       <x:c r="R160" s="2" t="str">
         <x:v>垂直末端主光线</x:v>
       </x:c>
+      <x:c r="S160" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G160))^2+TAN(RADIANS(H160))^2)))</x:f>
+        <x:v>7.499999999999999</x:v>
+      </x:c>
     </x:row>
     <x:row r="161" ht="24" customHeight="1">
       <x:c r="A161" s="24" t="n">
@@ -9732,6 +10351,10 @@
       <x:c r="R161" s="2" t="str">
         <x:v>垂直末端主光线</x:v>
       </x:c>
+      <x:c r="S161" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G161))^2+TAN(RADIANS(H161))^2)))</x:f>
+        <x:v>7.499999999999999</x:v>
+      </x:c>
     </x:row>
     <x:row r="162" ht="24" customHeight="1">
       <x:c r="A162" s="24" t="n">
@@ -9789,6 +10412,10 @@
       <x:c r="R162" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S162" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G162))^2+TAN(RADIANS(H162))^2)))</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="163" ht="24" customHeight="1">
       <x:c r="A163" s="24" t="n">
@@ -9846,6 +10473,10 @@
       <x:c r="R163" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S163" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G163))^2+TAN(RADIANS(H163))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="164" ht="24" customHeight="1">
       <x:c r="A164" s="24" t="n">
@@ -9903,6 +10534,10 @@
       <x:c r="R164" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S164" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G164))^2+TAN(RADIANS(H164))^2)))</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="165" ht="24" customHeight="1">
       <x:c r="A165" s="24" t="n">
@@ -9960,6 +10595,10 @@
       <x:c r="R165" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S165" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G165))^2+TAN(RADIANS(H165))^2)))</x:f>
+        <x:v>7.499999999999999</x:v>
+      </x:c>
     </x:row>
     <x:row r="166" ht="24" customHeight="1">
       <x:c r="A166" s="24" t="n">
@@ -10017,6 +10656,10 @@
       <x:c r="R166" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S166" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G166))^2+TAN(RADIANS(H166))^2)))</x:f>
+        <x:v>7.499999999999999</x:v>
+      </x:c>
     </x:row>
     <x:row r="167" ht="24" customHeight="1">
       <x:c r="A167" s="24" t="n">
@@ -10074,11 +10717,15 @@
       <x:c r="R167" s="2" t="str">
         <x:v>平行工件XY</x:v>
       </x:c>
+      <x:c r="S167" s="17" t="n">
+        <x:f>DEGREES(ATAN(SQRT(TAN(RADIANS(G167))^2+TAN(RADIANS(H167))^2)))</x:f>
+        <x:v>7.499999999999999</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8eae01bf814c4c81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dd90e0efcd14b5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>